<commit_message>
cleaned up scripts (moved to tests/legacy and tests/experimental) and solved R CMD checks failing
</commit_message>
<xml_diff>
--- a/inst/extdata/mocaredd-templatev2-simple.xlsx
+++ b/inst/extdata/mocaredd-templatev2-simple.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gaelsola/code/mocaredd.dev2/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{420F0AE4-D2D4-A04E-8681-F39E2EFA27D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1360EB88-E4CD-CB47-83D8-3D2645406C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="28200" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,7 +446,7 @@
     <t>C</t>
   </si>
   <si>
-    <t>NA</t>
+    <t>ratio</t>
   </si>
 </sst>
 </file>

</xml_diff>